<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.003-04 L'étoile et la feuille
Réécriture vocale example4 : éclat de platane, lunettes vécues.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.003-04.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.003-04.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>parc le matin, puis petite maison</t>
+          <t>parc sous les platanes, bac à feuilles, puis atelier (pâte, emporte-pièce)</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, Victorina, maman</t>
+          <t>Sarah, Victorina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut une étoile de pâte avec une vraie feuille dessus. La première feuille s'effrite. Victorina en trouve une souple. L'étoile repose sur l'assiette.</t>
+          <t>Un platane lâche un petit bruit, sec. Sur le bord du bac, un éclat de platane brille. Sarah veut une étoile avec une feuille, maintenant. Victorina arrive. Un rire commence. Victorina se tait. La feuille sèche casse. Sarah refuse de foncer. Elles portent la souple. Merci vécu. L'emporte-pièce trop vite. L'éclat de platane tient sur la manche.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le toboggan du parc a un peu de givre. Il est froid sous le doigt. Le souffle de Sarah fait un nuage. La petite maison sent le savon. Maman boutonne le gilet de Sarah. Le gilet est doux et épais. Un oiseau crie tout près. Tu es bien au chaud, Sarah ? Oui, maman. Tes mains sont froides. Un peu. On les frotte. Sarah frotte ses mains. Elles redeviennent tièdes. En ce moment, Sarah cherche une feuille. L'herbe sent la rosée. Je veux une étoile. Avec une feuille dessus. On la presse dans la pâte ? Oui. Une vraie nervure, alors. Victorina arrive près du toboggan. Victorina a des lunettes rondes. Elle a les cheveux tressés. Elle porte un gilet jaune. Victorina, tu cherches aussi. Tu m'aides, Victorina ? Oui. Sarah ramasse une feuille jaune. Elle est sèche et fragile. Elle s'effrite entre les doigts. Un peu de jaune reste sur la main. Elle casse. On en cherche une souple. Victorina se penche. Elle choisit une feuille molle. Celle-ci. Elle est encore molle.</t>
+          <t>Un platane lâche un petit bruit, sec. J'ai entendu, papa ! Tu as entendu le platane ? Oui, un petit bruit. Un éclat pâle glisse le long du tronc. Il brille, maman. Tu le vois, le petit point ? Oui, pâle. Il s'arrête sur le bord du bac. Sur le bord du bac, un éclat de platane brille. Le bac est froid, Sarah ? Un peu, papa. Le bac sent le platane, un peu humide. Tes mains sont froides, Sarah ? Un peu. On les frotte ? Oui. Sarah frotte ses mains. Elles redeviennent tièdes. En ce moment, Sarah cherche une feuille. Je veux une étoile, maintenant ! Avec une feuille dessus. On la presse dans la pâte ? Oui. Une vraie nervure, alors ? Oui, papa. Victorina arrive près du bac. Victorina a des lunettes rondes. Elle a les cheveux tressés. Elle porte un gilet jaune. Victorina, tu cherches aussi ? Tu m'aides, Victorina ? Oui. Sarah ramasse une feuille trop vite. La feuille est sèche et fragile. Elle s'effrite entre les doigts. Elle casse ! Sarah regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Victorina ne dit rien. Le sourire de Victorina disparaît. Tu la trouves, maintenant ! Non. Victorina recule d'un pas. Oh. Sarah veut presser toute seule. La feuille sèche tombe dans le bac. Ça fait un bruit mou. L'éclat de platane tremble, puis tient. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorina, Sarah ? Oui, papa. Tes mains sont collantes, Sarah ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le toboggan du parc a un peu de givre. Il est froid sous le doigt. Le souffle de Sarah fait un nuage. La petite maison sent le savon. Maman boutonne le gilet de Sarah. Le gilet est doux et épais. Un oiseau crie tout près. Tu es bien au chaud, Sarah ? Oui, maman. Tes mains sont froides. Un peu. On les frotte. Sarah frotte ses mains. Elles redeviennent tièdes. En ce moment, Sarah cherche une feuille. L'herbe sent la rosée. Je veux une étoile. Avec une feuille dessus. On la presse dans la pâte ? Oui. Une vraie nervure, alors. Victorina arrive près du toboggan. Victorina a des lunettes rondes. Elle a les cheveux tressés. Elle porte un gilet jaune. Victorina, tu cherches aussi. Tu m'aides, Victorina ? Oui. Sarah ramasse une feuille jaune. Elle est sèche et fragile. Elle s'effrite entre les doigts. Un peu de jaune reste sur la main. Elle casse. On en cherche une souple. Victorina se penche. Elle choisit une feuille molle. Celle-ci. Elle est encore molle.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un platane lâche un petit bruit, sec. J'ai entendu, papa ! Tu as entendu le platane ? Oui, un petit bruit. Un éclat pâle glisse le long du tronc. Il brille, maman. Tu le vois, le petit point ? Oui, pâle. Il s'arrête sur le bord du bac. Sur le bord du bac, un &lt;emphasis level="moderate"&gt;éclat de platane&lt;/emphasis&gt; brille. Le bac est froid, Sarah ? Un peu, papa. Le bac sent le platane, un peu humide. Tes mains sont froides, Sarah ? Un peu. On les frotte ? Oui. Sarah frotte ses mains. Elles redeviennent tièdes. En ce moment, Sarah cherche une feuille. Je veux une étoile, maintenant ! Avec une feuille dessus. On la presse dans la pâte ? Oui. Une vraie nervure, alors ? Oui, papa. Victorina arrive près du bac. Victorina a des lunettes rondes. Elle a les cheveux tressés. Elle porte un gilet jaune. Victorina, tu cherches aussi ? Tu m'aides, Victorina ? Oui. Sarah ramasse une feuille trop vite. La feuille est sèche et fragile. Elle s'effrite entre les doigts. Elle casse ! Sarah regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Victorina ne dit rien. Le sourire de Victorina disparaît. Tu la trouves, maintenant ! Non. Victorina recule d'un pas. Oh. Sarah veut presser toute seule. La feuille sèche tombe dans le bac. Ça fait un bruit mou. L'éclat de platane tremble, puis tient. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorina, Sarah ? Oui, papa. Tes mains sont collantes, Sarah ? Un peu, maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le matin, maman accompagne Océane au parc. L'herbe sent la rosée. Une amie arrive. Elle a des lunettes rondes. Elle a les cheveux tressés. Elle porte un gilet jaune. Océane regarde. Un autre enfant laisse sortir un petit rire. Maman s'approche tout de suite. Maman dit : on ne va &lt;emphasis&gt;pas&lt;/emphasis&gt; rire de l'apparence. Les lunettes aident à voir. Les cheveux sont les cheveux. L'habit tient chaud. On joue. Océane hoche la tête. Elle va vers l'amie. Océane dit : tu viens au bac à feuilles. Elles ramassent des feuilles. Plus tard, à l'atelier, il y a de la pâte. Océane se souvient. Un enfant regarde encore les lunettes. Océane dit : on ne va pas rire. On joue. Elles roulent la pâte. Les lunettes restent sur le nez. Les tresses bougent. Le gilet jaune reste boutonné. On ne rit pas des lunettes, des cheveux ou d'un habit. On ne va pas rire de l'apparence. On joue ensemble. [pause]</t>
+          <t>Un platane lâche un petit bruit, sec. J'ai entendu, papa ! Tu as entendu le platane ? Oui, un petit bruit. Un éclat pâle glisse le long du tronc. Il brille, maman. Tu le vois, le petit point ? Oui, pâle. Il s'arrête sur le bord du bac. Sur le bord du bac, un &lt;emphasis&gt;éclat de platane&lt;/emphasis&gt; brille. Le bac est froid, Sarah ? Un peu, papa. Le bac sent le platane, un peu humide. Tes mains sont froides, Sarah ? Un peu. On les frotte ? Oui. Sarah frotte ses mains. Elles redeviennent tièdes. En ce moment, Sarah cherche une feuille. Je veux une étoile, maintenant ! Avec une feuille dessus. On la presse dans la pâte ? Oui. Une vraie nervure, alors ? Oui, papa. Victorina arrive près du bac. Victorina a des lunettes rondes. Elle a les cheveux tressés. Elle porte un gilet jaune. Victorina, tu cherches aussi ? Tu m'aides, Victorina ? Oui. Sarah ramasse une feuille trop vite. La feuille est sèche et fragile. Elle s'effrite entre les doigts. Elle casse ! Sarah regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Victorina ne dit rien. Le sourire de Victorina disparaît. Tu la trouves, maintenant ! Non. Victorina recule d'un pas. Oh. Sarah veut presser toute seule. La feuille sèche tombe dans le bac. Ça fait un bruit mou. L'éclat de platane tremble, puis tient. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorina, Sarah ? Oui, papa. Tes mains sont collantes, Sarah ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>éclat de platane</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,47 +1321,70 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_l_etoile_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le toboggan du parc a un peu de givre.
-narrateur|Il est froid sous le doigt.
-narrateur|Le souffle de Sarah fait un nuage.
-narrateur|La petite maison sent le savon.
-narrateur|Maman boutonne le gilet de Sarah.
-narrateur|Le gilet est doux et épais.
-narrateur|Un oiseau crie tout près.
-maman|Tu es bien au chaud, Sarah ?
-enfant-f|Oui, maman.
-maman|Tes mains sont froides.
+          <t>narrateur|Un platane lâche un petit bruit, sec.
+enfant-f|J'ai entendu, papa !
+papa|Tu as entendu le platane ?
+enfant-f|Oui, un petit bruit.
+narrateur|Un éclat pâle glisse le long du tronc.
+enfant-f|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-f|Oui, pâle.
+narrateur|Il s'arrête sur le bord du bac.
+narrateur|Sur le bord du bac, un éclat de platane brille.
+papa|Le bac est froid, Sarah ?
+enfant-f|Un peu, papa.
+narrateur|Le bac sent le platane, un peu humide.
+maman|Tes mains sont froides, Sarah ?
 enfant-f|Un peu.
-maman|On les frotte.
+papa|On les frotte ?
+enfant-f|Oui.
 narrateur|Sarah frotte ses mains.
 narrateur|Elles redeviennent tièdes.
 narrateur|En ce moment, Sarah cherche une feuille.
-narrateur|L'herbe sent la rosée.
-enfant-f|Je veux une étoile.
+enfant-f|Je veux une étoile, maintenant !
 enfant-f|Avec une feuille dessus.
 maman|On la presse dans la pâte ?
 enfant-f|Oui.
-maman|Une vraie nervure, alors.
-narrateur|Victorina arrive près du toboggan.
+papa|Une vraie nervure, alors ?
+enfant-f|Oui, papa.
+narrateur|Victorina arrive près du bac.
 narrateur|Victorina a des lunettes rondes.
 narrateur|Elle a les cheveux tressés.
 narrateur|Elle porte un gilet jaune.
-maman|Victorina, tu cherches aussi.
+papa|Victorina, tu cherches aussi ?
 enfant-f|Tu m'aides, Victorina ?
 copine|Oui.
-narrateur|Sarah ramasse une feuille jaune.
-narrateur|Elle est sèche et fragile.
+narrateur|Sarah ramasse une feuille trop vite.
+narrateur|La feuille est sèche et fragile.
 narrateur|Elle s'effrite entre les doigts.
-narrateur|Un peu de jaune reste sur la main.
-enfant-f|Elle casse.
-maman|On en cherche une souple.
-narrateur|Victorina se penche.
-narrateur|Elle choisit une feuille molle.
-copine|Celle-ci.
-copine|Elle est encore molle.</t>
+enfant-f|Elle casse !
+narrateur|Sarah regarde les lunettes, trop longtemps.
+narrateur|Un rire commence dans sa bouche.
+narrateur|Victorina ne dit rien.
+narrateur|Le sourire de Victorina disparaît.
+enfant-f|Tu la trouves, maintenant !
+copine|Non.
+narrateur|Victorina recule d'un pas.
+enfant-f|Oh.
+narrateur|Sarah veut presser toute seule.
+narrateur|La feuille sèche tombe dans le bac.
+narrateur|Ça fait un bruit mou.
+narrateur|L'éclat de platane tremble, puis tient.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Victorina, Sarah ?
+enfant-f|Oui, papa.
+maman|Tes mains sont collantes, Sarah ?
+enfant-f|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1398,22 +1421,22 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorina a des lunettes. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorina a des &lt;emphasis level="moderate"&gt;lunettes&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>L'amie a des lunettes. Que fait-on ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorina a des &lt;emphasis&gt;lunettes&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>jouer</t>
+          <t>pas rire</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>jouer | ensemble | feuille | on joue | presser | pas rire</t>
+          <t>pas rire | on joue | jouer | pas rire apparence</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1466,7 +1489,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1474,10 +1497,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1492,34 +1515,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>lunettes</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1528,23 +1555,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=on_ne_rit_pas_victorina_a_des_lunettes; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1577,17 +1604,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend la feuille souple. Elle la pose dans sa main. Merci, Sarah. Merci, Victorina. On va à la petite maison ? Oui. La pâte nous attend. La table est froide et lisse. La pâte sent la farine. Elle colle un peu aux doigts. Victorina a trouvé la souple. On presse. Sarah fait un boudin. Victorina fait une boule. L'étoile. La feuille.</t>
+          <t>Sarah veut l'étoile, tout de suite. Je presse, maintenant ! Elle avance trop vite vers Victorina. Les mots se bousculent dans sa bouche. Non. Victorina reste un peu plus loin. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le bac, un instant. Elle écoute le petit bruit du platane. Tu veux l'étoile avec Victorina ? Papa reste à la même hauteur. Tu cherches avec moi ? Victorina ne dit rien, d'abord. Elle se penche sur le bac. Celle-ci. Elle est molle. D'accord. Merci, Sarah. Papa a vu les deux, près du bac. La feuille est souple, sous les doigts. Elle ne casse pas. Sarah pose la feuille dans sa main. Victorina reste plus près. On va à l'atelier ? Oui. La pâte nous attend. Tu portes la feuille, Sarah ? Oui, papa. Ils passent sous les platanes. Le gilet jaune bouge. Les tresses tapent le dos. Les lunettes restent sur le nez. La table, maman. Elle est froide et lisse. La pâte colle un peu aux doigts. On étale, sans se presser ? Oui. Sarah fait un boudin. Victorina fait une boule. L'étoile. La feuille. Tes mains sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend la feuille souple. Elle la pose dans sa main. Merci, Sarah. Merci, Victorina. On va à la petite maison ? Oui. La pâte nous attend. La table est froide et lisse. La pâte sent la farine. Elle colle un peu aux doigts. Victorina a trouvé la souple. On presse. Sarah fait un boudin. Victorina fait une boule. L'étoile. La feuille.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah veut l'étoile, tout de suite. Je presse, maintenant ! Elle avance trop vite vers Victorina. Les mots se bousculent dans sa bouche. Non. Victorina reste un peu plus loin. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le bac, un instant. Elle écoute le petit bruit du platane. Tu veux l'étoile avec Victorina ? Papa reste à la même hauteur. Tu cherches avec moi ? Victorina ne dit rien, d'abord. Elle se penche sur le bac. Celle-ci. Elle est molle. D'accord. Merci, Sarah. Papa a vu les deux, près du bac. La &lt;emphasis level="moderate"&gt;feuille&lt;/emphasis&gt; est souple, sous les doigts. Elle ne casse pas. Sarah pose la feuille dans sa main. Victorina reste plus près. On va à l'atelier ? Oui. La pâte nous attend. Tu portes la feuille, Sarah ? Oui, papa. Ils passent sous les platanes. Le gilet jaune bouge. Les tresses tapent le dos. Les lunettes restent sur le nez. La table, maman. Elle est froide et lisse. La pâte colle un peu aux doigts. On étale, sans se presser ? Oui. Sarah fait un boudin. Victorina fait une boule. L'étoile. La feuille. Tes mains sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Océane a entendu maman. On ne va &lt;emphasis&gt;pas&lt;/emphasis&gt; rire de l'apparence. Océane a invité l'amie. Elles ont joué. [pause]</t>
+          <t>Sarah veut l'étoile, tout de suite. Je presse, maintenant ! Elle avance trop vite vers Victorina. Les mots se bousculent dans sa bouche. Non. Victorina reste un peu plus loin. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le bac, un instant. Elle écoute le petit bruit du platane. Tu veux l'étoile avec Victorina ? Papa reste à la même hauteur. Tu cherches avec moi ? Victorina ne dit rien, d'abord. Elle se penche sur le bac. Celle-ci. Elle est molle. D'accord. Merci, Sarah. Papa a vu les deux, près du bac. La &lt;emphasis&gt;feuille&lt;/emphasis&gt; est souple, sous les doigts. Elle ne casse pas. Sarah pose la feuille dans sa main. Victorina reste plus près. On va à l'atelier ? Oui. La pâte nous attend. Tu portes la feuille, Sarah ? Oui, papa. Ils passent sous les platanes. Le gilet jaune bouge. Les tresses tapent le dos. Les lunettes restent sur le nez. La table, maman. Elle est froide et lisse. La pâte colle un peu aux doigts. On étale, sans se presser ? Oui. Sarah fait un boudin. Victorina fait une boule. L'étoile. La feuille. Tes mains sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1634,7 +1661,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1642,10 +1669,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1668,30 +1695,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>feuille</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1700,10 +1727,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1716,27 +1743,63 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elles_portent_la_feuille_a_deux; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah prend la feuille souple.
-narrateur|Elle la pose dans sa main.
-maman|Merci, Sarah.
-maman|Merci, Victorina.
-enfant-f|On va à la petite maison ?
+          <t>narrateur|Sarah veut l'étoile, tout de suite.
+enfant-f|Je presse, maintenant !
+narrateur|Elle avance trop vite vers Victorina.
+narrateur|Les mots se bousculent dans sa bouche.
+copine|Non.
+narrateur|Victorina reste un peu plus loin.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le bac, un instant.
+narrateur|Elle écoute le petit bruit du platane.
+papa|Tu veux l'étoile avec Victorina ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Tu cherches avec moi ?
+narrateur|Victorina ne dit rien, d'abord.
+narrateur|Elle se penche sur le bac.
+copine|Celle-ci.
+copine|Elle est molle.
+enfant-f|D'accord.
+papa|Merci, Sarah.
+narrateur|Papa a vu les deux, près du bac.
+maman|La feuille est souple, sous les doigts.
+enfant-f|Elle ne casse pas.
+narrateur|Sarah pose la feuille dans sa main.
+narrateur|Victorina reste plus près.
+enfant-f|On va à l'atelier ?
 maman|Oui.
 maman|La pâte nous attend.
-narrateur|La table est froide et lisse.
-narrateur|La pâte sent la farine.
-narrateur|Elle colle un peu aux doigts.
-maman|Victorina a trouvé la souple.
-maman|On presse.
+papa|Tu portes la feuille, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Ils passent sous les platanes.
+narrateur|Le gilet jaune bouge.
+narrateur|Les tresses tapent le dos.
+narrateur|Les lunettes restent sur le nez.
+enfant-f|La table, maman.
+maman|Elle est froide et lisse.
+narrateur|La pâte colle un peu aux doigts.
+papa|On étale, sans se presser ?
+enfant-f|Oui.
 narrateur|Sarah fait un boudin.
 narrateur|Victorina fait une boule.
 enfant-f|L'étoile.
-copine|La feuille.</t>
+copine|La feuille.
+maman|Tes mains sont au chaud ?
+enfant-f|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pate</t>
         </is>
       </c>
     </row>
@@ -1763,17 +1826,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah appuie l'emporte-pièce. L'étoile se dessine. Victorina pose la feuille. Sarah presse tout doux. La nervure s'imprime dans la pâte. Elle est restée ! On voit les traits. Bravo. Vous avez pressé ensemble. Un peu de farine tombe. Ça fait un nuage tout petit. Sarah souffle dessus, tout doux. Vous voulez laver les mains ? Oui. L'eau de la bassine est tiède. Sarah frotte. Victorina frotte. Elles posent l'étoile sur l'assiette. L'assiette est blanche et mate. Ma feuille est dessus. Oui. Elle est souple. On voit même les bords. Un peu de givre fond dehors.</t>
+          <t>Sarah prend l'emporte-pièce. Le métal est froid, un peu lourd. L'étoile, maintenant ! Elle appuie trop vite, tout de suite. Elle regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Victorina lâche le bord de la pâte. La feuille glisse sur le côté. Ça part ! Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la pâte, un instant. Elle écoute le petit bruit du platane. Sur la manche, un éclat de platane luit. Là, sur la manche. Tu poses la feuille, Victorina ? Victorina ne dit rien. Elle reprend le bord, sans parler. Oui. Sarah appuie, sans se presser. Victorina pose la feuille. La nervure s'imprime dans la pâte. Elle est restée ! On voit les traits. Tu as pressé sans t'arrêter ? Oui, papa. Le gilet est chaud, Victorina ? Un peu. Un peu de pâte tombe. Ça fait un nuage tout petit. On pose l'étoile ? Sur l'assiette. L'assiette est blanche et mate. Ma feuille est dessus. Oui. Elle est souple. On voit même les bords. La pâte a tenu, Sarah ? Oui, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah appuie l'emporte-pièce. L'étoile se dessine. Victorina pose la feuille. Sarah presse tout doux. La nervure s'imprime dans la pâte. Elle est restée ! On voit les traits. Bravo. Vous avez pressé ensemble. Un peu de farine tombe. Ça fait un nuage tout petit. Sarah souffle dessus, tout doux. Vous voulez laver les mains ? Oui. L'eau de la bassine est tiède. Sarah frotte. Victorina frotte. Elles posent l'étoile sur l'assiette. L'assiette est blanche et mate. Ma feuille est dessus. Oui. Elle est souple. On voit même les bords. Un peu de givre fond dehors.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah prend l'emporte-pièce. Le métal est froid, un peu lourd. L'étoile, maintenant ! Elle appuie trop vite, tout de suite. Elle regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Victorina lâche le bord de la pâte. La feuille glisse sur le côté. Ça part ! Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la pâte, un instant. Elle écoute le petit bruit du platane. Sur la manche, un &lt;emphasis level="moderate"&gt;éclat de platane&lt;/emphasis&gt; luit. Là, sur la manche. Tu poses la feuille, Victorina ? Victorina ne dit rien. Elle reprend le bord, sans parler. Oui. Sarah appuie, sans se presser. Victorina pose la feuille. La nervure s'imprime dans la pâte. Elle est restée ! On voit les traits. Tu as pressé sans t'arrêter ? Oui, papa. Le gilet est chaud, Victorina ? Un peu. Un peu de pâte tombe. Ça fait un nuage tout petit. On pose l'étoile ? Sur l'assiette. L'assiette est blanche et mate. Ma feuille est dessus. Oui. Elle est souple. On voit même les bords. La pâte a tenu, Sarah ? Oui, papa.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman revient près du portail. Océane et l'amie se disent à de&lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Sarah prend l'emporte-pièce. Le métal est froid, un peu lourd. L'étoile, maintenant ! Elle appuie trop vite, tout de suite. Elle regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Victorina lâche le bord de la pâte. La feuille glisse sur le côté. Ça part ! Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la pâte, un instant. Elle écoute le petit bruit du platane. Sur la manche, un &lt;emphasis&gt;éclat de platane&lt;/emphasis&gt; luit. Là, sur la manche. Tu poses la feuille, Victorina ? Victorina ne dit rien. Elle reprend le bord, sans parler. Oui. Sarah appuie, sans se presser. Victorina pose la feuille. La nervure s'imprime dans la pâte. Elle est restée ! On voit les traits. Tu as pressé sans t'arrêter ? Oui, papa. Le gilet est chaud, Victorina ? Un peu. Un peu de pâte tombe. Ça fait un nuage tout petit. On pose l'étoile ? Sur l'assiette. L'assiette est blanche et mate. Ma feuille est dessus. Oui. Elle est souple. On voit même les bords. La pâte a tenu, Sarah ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1820,7 +1883,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1828,10 +1891,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1854,30 +1917,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de platane</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1886,10 +1949,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1900,33 +1963,61 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sarah appuie l'emporte-pièce.
-narrateur|L'étoile se dessine.
+          <t>narrateur|Sarah prend l'emporte-pièce.
+narrateur|Le métal est froid, un peu lourd.
+enfant-f|L'étoile, maintenant !
+narrateur|Elle appuie trop vite, tout de suite.
+narrateur|Elle regarde les lunettes, trop longtemps.
+narrateur|Un rire revient dans sa bouche.
+copine|Attends.
+narrateur|Victorina lâche le bord de la pâte.
+narrateur|La feuille glisse sur le côté.
+enfant-f|Ça part !
+narrateur|Sarah avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Sarah refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe la pâte, un instant.
+narrateur|Elle écoute le petit bruit du platane.
+narrateur|Sur la manche, un éclat de platane luit.
+enfant-f|Là, sur la manche.
+enfant-f|Tu poses la feuille, Victorina ?
+narrateur|Victorina ne dit rien.
+narrateur|Elle reprend le bord, sans parler.
+copine|Oui.
+narrateur|Sarah appuie, sans se presser.
 narrateur|Victorina pose la feuille.
-narrateur|Sarah presse tout doux.
 narrateur|La nervure s'imprime dans la pâte.
 enfant-f|Elle est restée !
 copine|On voit les traits.
-maman|Bravo.
-maman|Vous avez pressé ensemble.
-narrateur|Un peu de farine tombe.
+papa|Tu as pressé sans t'arrêter ?
+enfant-f|Oui, papa.
+maman|Le gilet est chaud, Victorina ?
+copine|Un peu.
+narrateur|Un peu de pâte tombe.
 narrateur|Ça fait un nuage tout petit.
-narrateur|Sarah souffle dessus, tout doux.
-maman|Vous voulez laver les mains ?
-enfant-f|Oui.
-narrateur|L'eau de la bassine est tiède.
-narrateur|Sarah frotte.
-narrateur|Victorina frotte.
-narrateur|Elles posent l'étoile sur l'assiette.
+papa|On pose l'étoile ?
+copine|Sur l'assiette.
 narrateur|L'assiette est blanche et mate.
 enfant-f|Ma feuille est dessus.
 maman|Oui.
 maman|Elle est souple.
 copine|On voit même les bords.
-narrateur|Un peu de givre fond dehors.</t>
+papa|La pâte a tenu, Sarah ?
+enfant-f|Oui, papa.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>pate</t>
         </is>
       </c>
     </row>
@@ -1953,17 +2044,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'étoile repose sur l'assiette. La feuille jaune est bien pressée. On l'a faite. Oui. Vous avez pressé l'étoile. Le givre fond sur le toboggan.</t>
+          <t>Ils restent près de la table. Maman essuie un peu de pâte. On a eu l'étoile, papa. Tu l'as vue, toi ? Oui, avec la feuille. On est bien, ici. Sarah tapote l'étoile du doigt. Elle a une trace de nervure. Tu la vois, la trace ? Oui, maman. L'étoile est restée, Sarah. Oui, avec Victorina. L'étoile est restée. Ça sent le platane, un peu tiède. Et la pâte, maman. Oui, dans l'air. La feuille reste sur l'étoile. Un éclat de platane tient sur la manche.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>L'étoile repose sur l'assiette. La feuille jaune est bien pressée. On l'a faite. Oui. Vous avez pressé l'étoile. Le givre fond sur le toboggan.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. Maman essuie un peu de pâte. On a eu l'étoile, papa. Tu l'as vue, toi ? Oui, avec la feuille. On est bien, ici. Sarah tapote l'étoile du doigt. Elle a une trace de nervure. Tu la vois, la trace ? Oui, maman. L'étoile est restée, Sarah. Oui, avec Victorina. L'étoile est restée. Ça sent le platane, un peu tiède. Et la pâte, maman. Oui, dans l'air. La feuille reste sur l'étoile. Un &lt;emphasis level="moderate"&gt;éclat de platane&lt;/emphasis&gt; tient sur la manche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. Maman essuie un peu de pâte. On a eu l'étoile, papa. Tu l'as vue, toi ? Oui, avec la feuille. On est bien, ici. Sarah tapote l'étoile du doigt. Elle a une trace de nervure. Tu la vois, la trace ? Oui, maman. L'étoile est restée, Sarah. Oui, avec Victorina. L'étoile est restée. Ça sent le platane, un peu tiède. Et la pâte, maman. Oui, dans l'air. La feuille reste sur l'étoile. Un &lt;emphasis&gt;éclat de platane&lt;/emphasis&gt; tient sur la manche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2010,18 +2101,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2030,12 +2121,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2044,17 +2135,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de platane</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2063,11 +2158,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2076,29 +2171,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_manche; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'étoile repose sur l'assiette.
-narrateur|La feuille jaune est bien pressée.
-enfant-f|On l'a faite.
-maman|Oui.
-maman|Vous avez pressé l'étoile.
-narrateur|Le givre fond sur le toboggan.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|Maman essuie un peu de pâte.
+enfant-f|On a eu l'étoile, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, avec la feuille.
+maman|On est bien, ici.
+narrateur|Sarah tapote l'étoile du doigt.
+enfant-f|Elle a une trace de nervure.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|L'étoile est restée, Sarah.
+enfant-f|Oui, avec Victorina.
+copine|L'étoile est restée.
+narrateur|Ça sent le platane, un peu tiède.
+enfant-f|Et la pâte, maman.
+maman|Oui, dans l'air.
+narrateur|La feuille reste sur l'étoile.
+narrateur|Un éclat de platane tient sur la manche.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pate</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2204,6 +2320,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>